<commit_message>
Task 1: DVC init + track synthetic dataset
- dvc init (analytics off); dvc add data/synthetic/demand.parquet -> pointer
  demand.parquet.dvc committed to git, 1.4MB parquet stays out of git
- add 'data' extra (dvc) to pyproject + make setup; new 'make data' target
  (regenerate + dvc add); README note; Task1_Summary checklist -> DVC done
- no remote yet (local versioning); a non-Apple remote can be added later
</commit_message>
<xml_diff>
--- a/docs/Task1_Summary.xlsx
+++ b/docs/Task1_Summary.xlsx
@@ -941,17 +941,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Remaining sub-step</t>
+          <t>Data versioning</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>DVC init + track the dataset with a remote.</t>
+          <t>DVC initialised; dataset tracked via demand.parquet.dvc (pointer in git, data out).</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Task 1 (pending)</t>
+          <t>dvc add / .dvc/</t>
         </is>
       </c>
     </row>
@@ -1571,14 +1571,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>DVC init + track dataset</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
         </is>
       </c>
     </row>

</xml_diff>